<commit_message>
Fixtures and tests use made-up prefixes, numbers and titles
The old codes (MATH, STAT, DATA, CS, CORE, EDUC, ASC) become MUSC, URBS,
DIGI, CRUD, BHAV, HELP and AMUS, which keeps their alphabetical order.
Course numbers in the fixtures move up by three; titles are invented.
The legacy workbooks and the derived fixture files are regenerated.

Assisted by Claude Sonnet 5.5 (Anthropic).
</commit_message>
<xml_diff>
--- a/fixtures/legacy/old-app-export.xlsx
+++ b/fixtures/legacy/old-app-export.xlsx
@@ -144,10 +144,10 @@
     <t>Mathematics and Statistics</t>
   </si>
   <si>
-    <t>MATH</t>
-  </si>
-  <si>
-    <t>101</t>
+    <t>MUSC</t>
+  </si>
+  <si>
+    <t>104</t>
   </si>
   <si>
     <t>A</t>
@@ -165,7 +165,7 @@
     <t>NH 101</t>
   </si>
   <si>
-    <t>Calculus I</t>
+    <t>Musical Patterns I</t>
   </si>
   <si>
     <t>Lecture</t>
@@ -177,7 +177,7 @@
     <t>In-Person</t>
   </si>
   <si>
-    <t>102</t>
+    <t>105</t>
   </si>
   <si>
     <t>11:00:00</t>
@@ -186,10 +186,10 @@
     <t>NH 102</t>
   </si>
   <si>
-    <t>Calculus II</t>
-  </si>
-  <si>
-    <t>231</t>
+    <t>Musical Patterns II</t>
+  </si>
+  <si>
+    <t>234</t>
   </si>
   <si>
     <t>TR</t>
@@ -201,16 +201,16 @@
     <t>NH 103</t>
   </si>
   <si>
-    <t>Linear Algebra</t>
+    <t>Harmonic Structures</t>
   </si>
   <si>
     <t>200</t>
   </si>
   <si>
-    <t>STAT</t>
-  </si>
-  <si>
-    <t>143</t>
+    <t>URBS</t>
+  </si>
+  <si>
+    <t>146</t>
   </si>
   <si>
     <t>12:15:00</t>
@@ -219,19 +219,19 @@
     <t>NH 105</t>
   </si>
   <si>
-    <t>Introduction to Statistics</t>
-  </si>
-  <si>
-    <t>243</t>
-  </si>
-  <si>
-    <t>Statistical Methods</t>
-  </si>
-  <si>
-    <t>DATA</t>
-  </si>
-  <si>
-    <t>202</t>
+    <t>Introduction to Behavioral Dynamics</t>
+  </si>
+  <si>
+    <t>246</t>
+  </si>
+  <si>
+    <t>Behavioral Methods</t>
+  </si>
+  <si>
+    <t>DIGI</t>
+  </si>
+  <si>
+    <t>205</t>
   </si>
   <si>
     <t>Fay Mockson</t>
@@ -243,16 +243,16 @@
     <t>SB 110</t>
   </si>
   <si>
-    <t>Data Computing</t>
+    <t>Information Computing</t>
   </si>
   <si>
     <t>Hybrid</t>
   </si>
   <si>
-    <t>CS</t>
-  </si>
-  <si>
-    <t>108</t>
+    <t>CRUD</t>
+  </si>
+  <si>
+    <t>111</t>
   </si>
   <si>
     <t>Gus Testwell</t>
@@ -261,7 +261,7 @@
     <t>SB 120</t>
   </si>
   <si>
-    <t>Introduction to Computing</t>
+    <t>Introduction to Urban Systems</t>
   </si>
   <si>
     <t>HNRS</t>
@@ -294,13 +294,13 @@
     <t>The registrar assigns the letter</t>
   </si>
   <si>
-    <t>232</t>
-  </si>
-  <si>
-    <t>Multivariable Calculus</t>
-  </si>
-  <si>
-    <t>302</t>
+    <t>235</t>
+  </si>
+  <si>
+    <t>Multivoice Analysis</t>
+  </si>
+  <si>
+    <t>305</t>
   </si>
   <si>
     <t>14:10:00</t>
@@ -309,13 +309,13 @@
     <t>NH 104</t>
   </si>
   <si>
-    <t>Real Analysis II</t>
+    <t>Corpus Studies II</t>
   </si>
   <si>
     <t>300</t>
   </si>
   <si>
-    <t>391</t>
+    <t>394</t>
   </si>
   <si>
     <t xml:space="preserve">R
@@ -336,13 +336,13 @@
     <t>Colloquium</t>
   </si>
   <si>
-    <t>244</t>
-  </si>
-  <si>
-    <t>Regression Models</t>
-  </si>
-  <si>
-    <t>301</t>
+    <t>247</t>
+  </si>
+  <si>
+    <t>Models of Change</t>
+  </si>
+  <si>
+    <t>304</t>
   </si>
   <si>
     <t>Fay Mockson, Ben Sample</t>
@@ -351,13 +351,13 @@
     <t>MW</t>
   </si>
   <si>
-    <t>Data Science Topics</t>
+    <t>Digital Information Topics</t>
   </si>
   <si>
     <t>Online (synchronous)</t>
   </si>
   <si>
-    <t>262</t>
+    <t>265</t>
   </si>
   <si>
     <t>Hal Fakename</t>
@@ -369,7 +369,7 @@
     <t>SB 122</t>
   </si>
   <si>
-    <t>Data Structures</t>
+    <t>Urban Data Structures</t>
   </si>
   <si>
     <t>StudentCredits</t>

</xml_diff>